<commit_message>
implements employee rank and grade data
</commit_message>
<xml_diff>
--- a/api/public/template/TEMPLATE-IMPOR-PEGAWAI.xlsx
+++ b/api/public/template/TEMPLATE-IMPOR-PEGAWAI.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="pangkat_golongan" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,8 +27,74 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Adnan Zaki</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>Adnan Zaki:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">
+Silakan cek sheet </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">“pangkat_golongan” </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve">kolom </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t>“A”</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="0"/>
+          </rPr>
+          <t xml:space="preserve"> untuk mengisi kolom ini</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t>nama</t>
   </si>
@@ -35,6 +102,9 @@
     <t>nip</t>
   </si>
   <si>
+    <t>pangkat_golongan_id</t>
+  </si>
+  <si>
     <t>jabatan</t>
   </si>
   <si>
@@ -48,6 +118,143 @@
   </si>
   <si>
     <t>PERHATIAN: Kolom jenis pegawai hanya boleh diisi dengan PNS, PPPK atau HONORER</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Silakan cek sheet </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">“pangkat_golongan” </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">kolom </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>“A”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> untuk mengisi kolom ini</t>
+    </r>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Jabatan</t>
+  </si>
+  <si>
+    <t>Jenis Pegawai</t>
+  </si>
+  <si>
+    <t>Juru Muda / I a</t>
+  </si>
+  <si>
+    <t>PNS</t>
+  </si>
+  <si>
+    <t>Juru Muda Tk. I / I b</t>
+  </si>
+  <si>
+    <t>Juru / I c</t>
+  </si>
+  <si>
+    <t>Juru Tk. I / I d</t>
+  </si>
+  <si>
+    <t>Pengatur Muda / II a</t>
+  </si>
+  <si>
+    <t>Pengatur Muda Tk. I / II b</t>
+  </si>
+  <si>
+    <t>Pengatur / II c</t>
+  </si>
+  <si>
+    <t>Pengatur Tk. I / II d</t>
+  </si>
+  <si>
+    <t>Penata Muda / III a</t>
+  </si>
+  <si>
+    <t>Penata Muda Tk. I / III b</t>
+  </si>
+  <si>
+    <t>Penata / III c</t>
+  </si>
+  <si>
+    <t>Penata Tk. I / III d</t>
+  </si>
+  <si>
+    <t>Pembina / IV a</t>
+  </si>
+  <si>
+    <t>Pembina Tk. I / IV b</t>
+  </si>
+  <si>
+    <t>Pembina Utama Muda / IV c</t>
+  </si>
+  <si>
+    <t>Pembina Utama Madya / IV d</t>
+  </si>
+  <si>
+    <t>Pembina Utama / IV e</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>PPPK</t>
+  </si>
+  <si>
+    <t>IV</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>VI</t>
+  </si>
+  <si>
+    <t>VII</t>
+  </si>
+  <si>
+    <t>IX</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>XI</t>
   </si>
 </sst>
 </file>
@@ -60,7 +267,7 @@
     <numFmt numFmtId="178" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="179" formatCode="_-&quot;Rp&quot;* #,##0_-;\-&quot;Rp&quot;* #,##0_-;_-&quot;Rp&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,13 +427,30 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="0"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -559,7 +783,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -583,16 +807,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -601,96 +825,111 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -701,12 +940,12 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -968,17 +1207,10 @@
 </styleSheet>
 </file>
 
-<file path=xl/customStorage/customStorage.xml><?xml version="1.0" encoding="utf-8"?>
-<customStorage xmlns="https://web.wps.cn/et/2018/main">
-  <book/>
-  <sheets/>
-</customStorage>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="WPS">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="WPS">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -992,40 +1224,40 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4874CB"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="EE822F"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="F2BA02"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="75BD42"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="30C0B4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="E54C5E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0026E5"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="7E1FAD"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="WPS">
       <a:majorFont>
         <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Arab" typeface="Traditional Arabic"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
         <a:font script="Ethi" typeface="Nyala"/>
@@ -1056,11 +1288,11 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
         <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Arab" typeface="Traditional Arabic"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
         <a:font script="Ethi" typeface="Nyala"/>
@@ -1088,66 +1320,40 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="WPS">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:lumOff val="17500"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
-              </a:schemeClr>
+              <a:schemeClr val="phClr"/>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="2700000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:hueOff val="-2520000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
-              </a:schemeClr>
+              <a:schemeClr val="phClr"/>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="2700000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1161,20 +1367,38 @@
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:gradFill>
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="phClr">
+                  <a:hueOff val="-4200000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="phClr"/>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="2700000" scaled="1"/>
+          </a:gradFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="101600" dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:schemeClr val="phClr">
+                <a:alpha val="60000"/>
+              </a:schemeClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:reflection stA="50000" endA="300" endPos="40000" dist="25400" dir="5400000" sy="-100000" algn="bl" rotWithShape="0"/>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
@@ -1232,65 +1456,364 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="21.7777777777778" customWidth="1"/>
+    <col min="1" max="1" width="15.5555555555556" customWidth="1"/>
     <col min="2" max="2" width="20.8888888888889" customWidth="1"/>
-    <col min="3" max="3" width="10.2222222222222" customWidth="1"/>
-    <col min="4" max="4" width="13.5555555555556" customWidth="1"/>
-    <col min="5" max="5" width="20.4444444444444" customWidth="1"/>
-    <col min="6" max="6" width="14.1111111111111" customWidth="1"/>
-    <col min="7" max="7" width="73" customWidth="1"/>
+    <col min="3" max="3" width="20.1111111111111" customWidth="1"/>
+    <col min="4" max="4" width="10.2222222222222" customWidth="1"/>
+    <col min="5" max="5" width="13.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="16.4444444444444" customWidth="1"/>
+    <col min="8" max="8" width="81.4444444444444" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" ht="57.6" spans="1:8">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="2"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="4Z+73pVGbnZLK9EHNAhhsrtt9pu+lH+0vxAuxWJLmjdls+NNrjwzjyNtQOX/uaIs0hSnIx/uWOs9JA0LAJR4GA==" saltValue="RF3VB3ePSba58SLWQNsgGg==" spinCount="100000" sheet="1" objects="1"/>
-  <protectedRanges>
-    <protectedRange sqref="A2:F500" name="input data"/>
-  </protectedRanges>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="8.88888888888889" style="1"/>
+    <col min="2" max="2" width="27.4444444444444" style="2" customWidth="1"/>
+    <col min="3" max="3" width="19" style="2" customWidth="1"/>
+    <col min="4" max="16384" width="8.88888888888889" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" spans="1:3">
+      <c r="A1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<allowEditUser xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main" hasInvisiblePropRange="0">
-  <rangeList sheetStid="1" master="" otherUserPermission="visible">
-    <arrUserId title="input data" rangeCreator="" othersAccessPermission="edit"/>
-  </rangeList>
-</allowEditUser>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5A5607D9-04D2-4DE1-AC0E-A7772F01BC71}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="https://web.wps.cn/et/2018/main"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>